<commit_message>
segmented serial version done
</commit_message>
<xml_diff>
--- a/run_data/numba_thread_sweep_ANALYSED.xlsx
+++ b/run_data/numba_thread_sweep_ANALYSED.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FMI\semester_2\Parallel_Programming_Python\primes\run_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AA26FC1-AB7B-4966-B7A5-F6B6885E06D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{D4BED7BD-B54F-4D82-B167-589C30EB1FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="17">
   <si>
     <t>function</t>
   </si>
@@ -71,11 +71,20 @@
   <si>
     <t>2026-07-03T18-25-00</t>
   </si>
+  <si>
+    <t>2026-07-05T06-32-26</t>
+  </si>
+  <si>
+    <t>N:</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="0E+00"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -553,9 +562,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -721,7 +734,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$20:$D$23</c:f>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$21:$D$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -742,7 +755,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'numba_thread_sweep_2026-07-03T1'!$E$20:$E$23</c:f>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$E$21:$E$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -800,7 +813,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$20:$D$23</c:f>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$21:$D$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -821,7 +834,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'numba_thread_sweep_2026-07-03T1'!$F$20:$F$23</c:f>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$F$21:$F$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -879,7 +892,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$20:$D$23</c:f>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$21:$D$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -900,7 +913,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'numba_thread_sweep_2026-07-03T1'!$G$20:$G$23</c:f>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$G$21:$G$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -958,7 +971,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$20:$D$23</c:f>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$21:$D$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -979,7 +992,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'numba_thread_sweep_2026-07-03T1'!$H$20:$H$23</c:f>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$H$21:$H$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -994,6 +1007,666 @@
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>1.3254532729999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-7593-4812-895A-1E9621077CB9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="750342064"/>
+        <c:axId val="750341648"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="750342064"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="8"/>
+          <c:min val="1"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>cores</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="750341648"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="750341648"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="1"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="750342064"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Speedup as a function of cores</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>1GB</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$30:$D$37</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$G$30:$G$37</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.4808839770204301</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.49284059768407</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.4519555200237899</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.47159213765737</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.5419937227326399</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.67317715074572</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.86269965911916</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-7593-4812-895A-1E9621077CB9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>100MB</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$30:$D$37</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$F$30:$F$37</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.34503978187853</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.251675085342</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.4146769288790499</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.3971630534516299</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.30930244822502</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.24161427510124</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.2940569898505301</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-7593-4812-895A-1E9621077CB9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>10MB</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$D$30:$D$37</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'numba_thread_sweep_2026-07-03T1'!$E$30:$E$37</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.4471576087676301</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.3590038479117601</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.36643995178902</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.1113363035288</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.2128101034236201</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.1042370185685799</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.0084406855250101</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1321,6 +1994,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1837,20 +2550,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
+      <xdr:col>19</xdr:col>
       <xdr:colOff>323850</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1870,6 +3099,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>428625</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC3A2A29-75AB-4169-B319-D251836F1EE7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2175,7 +3440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.140625" bestFit="1" customWidth="1"/>
@@ -2929,8 +4194,8 @@
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="D19" t="s">
-        <v>1</v>
+      <c r="D19" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="E19">
         <f>B2</f>
@@ -2950,71 +4215,1066 @@
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="E20">
-        <v>1</v>
-      </c>
-      <c r="F20">
-        <v>1</v>
-      </c>
-      <c r="G20">
-        <v>1</v>
-      </c>
-      <c r="H20">
-        <v>1</v>
-      </c>
+      <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21">
-        <v>1.4138100069999999</v>
+        <v>1</v>
       </c>
       <c r="F21">
-        <v>1.42358362</v>
+        <v>1</v>
       </c>
       <c r="G21">
-        <v>1.03514459</v>
+        <v>1</v>
       </c>
       <c r="H21">
-        <v>1.4234428859999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D22">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E22">
-        <v>1.7879426860000001</v>
+        <v>1.4138100069999999</v>
       </c>
       <c r="F22">
-        <v>1.6875924229999999</v>
+        <v>1.42358362</v>
       </c>
       <c r="G22">
-        <v>1.529290875</v>
+        <v>1.03514459</v>
       </c>
       <c r="H22">
-        <v>1.7847859239999999</v>
+        <v>1.4234428859999999</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D23">
+        <v>4</v>
+      </c>
+      <c r="E23">
+        <v>1.7879426860000001</v>
+      </c>
+      <c r="F23">
+        <v>1.6875924229999999</v>
+      </c>
+      <c r="G23">
+        <v>1.529290875</v>
+      </c>
+      <c r="H23">
+        <v>1.7847859239999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D24">
         <v>8</v>
       </c>
-      <c r="E23">
+      <c r="E24">
         <v>1.6968358830000001</v>
       </c>
-      <c r="F23">
+      <c r="F24">
         <v>1.6618190070000001</v>
       </c>
-      <c r="G23">
+      <c r="G24">
         <v>1.8206657939999999</v>
       </c>
-      <c r="H23">
+      <c r="H24">
         <v>1.3254532729999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="3">
+        <v>10000000</v>
+      </c>
+      <c r="F28" s="3">
+        <v>100000000</v>
+      </c>
+      <c r="G28">
+        <v>1000000000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D30">
+        <v>1</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30">
+        <v>1</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="E31">
+        <v>1.4471576087676301</v>
+      </c>
+      <c r="F31">
+        <v>1.34503978187853</v>
+      </c>
+      <c r="G31">
+        <v>1.4808839770204301</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D32">
+        <v>3</v>
+      </c>
+      <c r="E32">
+        <v>1.3590038479117601</v>
+      </c>
+      <c r="F32">
+        <v>1.251675085342</v>
+      </c>
+      <c r="G32">
+        <v>1.49284059768407</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D33">
+        <v>4</v>
+      </c>
+      <c r="E33">
+        <v>1.36643995178902</v>
+      </c>
+      <c r="F33">
+        <v>1.4146769288790499</v>
+      </c>
+      <c r="G33">
+        <v>1.4519555200237899</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D34">
+        <v>5</v>
+      </c>
+      <c r="E34">
+        <v>1.1113363035288</v>
+      </c>
+      <c r="F34">
+        <v>1.3971630534516299</v>
+      </c>
+      <c r="G34">
+        <v>1.47159213765737</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D35">
+        <v>6</v>
+      </c>
+      <c r="E35">
+        <v>1.2128101034236201</v>
+      </c>
+      <c r="F35">
+        <v>1.30930244822502</v>
+      </c>
+      <c r="G35">
+        <v>1.5419937227326399</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D36">
+        <v>7</v>
+      </c>
+      <c r="E36">
+        <v>1.1042370185685799</v>
+      </c>
+      <c r="F36">
+        <v>1.24161427510124</v>
+      </c>
+      <c r="G36">
+        <v>1.67317715074572</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D37">
+        <v>8</v>
+      </c>
+      <c r="E37">
+        <v>1.0084406855250101</v>
+      </c>
+      <c r="F37">
+        <v>1.2940569898505301</v>
+      </c>
+      <c r="G37">
+        <v>1.86269965911916</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>0</v>
+      </c>
+      <c r="B41" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>2</v>
+      </c>
+      <c r="D41" t="s">
+        <v>3</v>
+      </c>
+      <c r="E41" t="s">
+        <v>4</v>
+      </c>
+      <c r="F41" t="s">
+        <v>5</v>
+      </c>
+      <c r="G41" t="s">
+        <v>6</v>
+      </c>
+      <c r="H41" t="s">
+        <v>8</v>
+      </c>
+      <c r="I41" t="s">
+        <v>9</v>
+      </c>
+      <c r="J41" t="s">
+        <v>10</v>
+      </c>
+      <c r="K41" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42">
+        <v>10000000</v>
+      </c>
+      <c r="C42">
+        <v>1</v>
+      </c>
+      <c r="D42" t="s">
+        <v>15</v>
+      </c>
+      <c r="E42">
+        <v>3.0999466670133698E-2</v>
+      </c>
+      <c r="F42">
+        <v>6.0055427123116402E-3</v>
+      </c>
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="H42">
+        <v>2.5638400009483999E-2</v>
+      </c>
+      <c r="I42">
+        <v>3.7489299997105201E-2</v>
+      </c>
+      <c r="J42">
+        <v>2.9870700003811999E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>13</v>
+      </c>
+      <c r="B43">
+        <v>10000000</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43" t="s">
+        <v>15</v>
+      </c>
+      <c r="E43">
+        <v>2.1420933340171599E-2</v>
+      </c>
+      <c r="F43">
+        <v>1.3918699498118501E-3</v>
+      </c>
+      <c r="G43">
+        <v>1.4471576087676301</v>
+      </c>
+      <c r="H43">
+        <v>2.2973700004513299E-2</v>
+      </c>
+      <c r="I43">
+        <v>2.1003700006985999E-2</v>
+      </c>
+      <c r="J43">
+        <v>2.0285400009015499E-2</v>
+      </c>
+      <c r="K43">
+        <v>3.0999466670133698E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>13</v>
+      </c>
+      <c r="B44">
+        <v>10000000</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44" t="s">
+        <v>15</v>
+      </c>
+      <c r="E44">
+        <v>2.2810433331566501E-2</v>
+      </c>
+      <c r="F44">
+        <v>3.6746247694999E-3</v>
+      </c>
+      <c r="G44">
+        <v>1.3590038479117601</v>
+      </c>
+      <c r="H44">
+        <v>2.15991000004578E-2</v>
+      </c>
+      <c r="I44">
+        <v>1.9894400000339301E-2</v>
+      </c>
+      <c r="J44">
+        <v>2.69377999939024E-2</v>
+      </c>
+      <c r="K44">
+        <v>3.0999466670133698E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45">
+        <v>10000000</v>
+      </c>
+      <c r="C45">
+        <v>4</v>
+      </c>
+      <c r="D45" t="s">
+        <v>15</v>
+      </c>
+      <c r="E45">
+        <v>2.26862999940446E-2</v>
+      </c>
+      <c r="F45">
+        <v>1.5268044041951299E-3</v>
+      </c>
+      <c r="G45">
+        <v>1.36643995178902</v>
+      </c>
+      <c r="H45">
+        <v>2.2610699990764201E-2</v>
+      </c>
+      <c r="I45">
+        <v>2.1198699992964899E-2</v>
+      </c>
+      <c r="J45">
+        <v>2.4249499998404599E-2</v>
+      </c>
+      <c r="K45">
+        <v>3.0999466670133698E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>13</v>
+      </c>
+      <c r="B46">
+        <v>10000000</v>
+      </c>
+      <c r="C46">
+        <v>5</v>
+      </c>
+      <c r="D46" t="s">
+        <v>15</v>
+      </c>
+      <c r="E46">
+        <v>2.7893866664574701E-2</v>
+      </c>
+      <c r="F46">
+        <v>7.5261150812572499E-3</v>
+      </c>
+      <c r="G46">
+        <v>1.1113363035288</v>
+      </c>
+      <c r="H46">
+        <v>3.6575899997842498E-2</v>
+      </c>
+      <c r="I46">
+        <v>2.3222500007250301E-2</v>
+      </c>
+      <c r="J46">
+        <v>2.38831999886315E-2</v>
+      </c>
+      <c r="K46">
+        <v>3.0999466670133698E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47">
+        <v>10000000</v>
+      </c>
+      <c r="C47">
+        <v>6</v>
+      </c>
+      <c r="D47" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47">
+        <v>2.5560033333022099E-2</v>
+      </c>
+      <c r="F47">
+        <v>2.9344889576068201E-3</v>
+      </c>
+      <c r="G47">
+        <v>1.2128101034236201</v>
+      </c>
+      <c r="H47">
+        <v>2.5970300004701099E-2</v>
+      </c>
+      <c r="I47">
+        <v>2.2442000001319601E-2</v>
+      </c>
+      <c r="J47">
+        <v>2.82677999930456E-2</v>
+      </c>
+      <c r="K47">
+        <v>3.0999466670133698E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48">
+        <v>10000000</v>
+      </c>
+      <c r="C48">
+        <v>7</v>
+      </c>
+      <c r="D48" t="s">
+        <v>15</v>
+      </c>
+      <c r="E48">
+        <v>2.8073200000411198E-2</v>
+      </c>
+      <c r="F48">
+        <v>4.1819575833571699E-3</v>
+      </c>
+      <c r="G48">
+        <v>1.1042370185685799</v>
+      </c>
+      <c r="H48">
+        <v>3.28898000007029E-2</v>
+      </c>
+      <c r="I48">
+        <v>2.5963299995055401E-2</v>
+      </c>
+      <c r="J48">
+        <v>2.53665000054752E-2</v>
+      </c>
+      <c r="K48">
+        <v>3.0999466670133698E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49">
+        <v>10000000</v>
+      </c>
+      <c r="C49">
+        <v>8</v>
+      </c>
+      <c r="D49" t="s">
+        <v>15</v>
+      </c>
+      <c r="E49">
+        <v>3.07399999971191E-2</v>
+      </c>
+      <c r="F49">
+        <v>3.0451500293367699E-3</v>
+      </c>
+      <c r="G49">
+        <v>1.0084406855250101</v>
+      </c>
+      <c r="H49">
+        <v>2.7297199994791299E-2</v>
+      </c>
+      <c r="I49">
+        <v>3.1842299998970702E-2</v>
+      </c>
+      <c r="J49">
+        <v>3.3080499997595297E-2</v>
+      </c>
+      <c r="K49">
+        <v>3.0999466670133698E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>13</v>
+      </c>
+      <c r="B50">
+        <v>100000000</v>
+      </c>
+      <c r="C50">
+        <v>1</v>
+      </c>
+      <c r="D50" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50">
+        <v>0.629853166668908</v>
+      </c>
+      <c r="F50">
+        <v>4.1548708403359299E-3</v>
+      </c>
+      <c r="G50">
+        <v>1</v>
+      </c>
+      <c r="H50">
+        <v>0.63457360000757002</v>
+      </c>
+      <c r="I50">
+        <v>0.62675060000037697</v>
+      </c>
+      <c r="J50">
+        <v>0.62823529999877703</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>13</v>
+      </c>
+      <c r="B51">
+        <v>100000000</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51" t="s">
+        <v>15</v>
+      </c>
+      <c r="E51">
+        <v>0.46827846667050199</v>
+      </c>
+      <c r="F51">
+        <v>9.2556291682539208E-3</v>
+      </c>
+      <c r="G51">
+        <v>1.34503978187853</v>
+      </c>
+      <c r="H51">
+        <v>0.45878359999915103</v>
+      </c>
+      <c r="I51">
+        <v>0.46877710000262501</v>
+      </c>
+      <c r="J51">
+        <v>0.47727470000972899</v>
+      </c>
+      <c r="K51">
+        <v>0.629853166668908</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>13</v>
+      </c>
+      <c r="B52">
+        <v>100000000</v>
+      </c>
+      <c r="C52">
+        <v>3</v>
+      </c>
+      <c r="D52" t="s">
+        <v>15</v>
+      </c>
+      <c r="E52">
+        <v>0.50320819999130095</v>
+      </c>
+      <c r="F52">
+        <v>6.7869265198035406E-2</v>
+      </c>
+      <c r="G52">
+        <v>1.251675085342</v>
+      </c>
+      <c r="H52">
+        <v>0.490758899992215</v>
+      </c>
+      <c r="I52">
+        <v>0.44242539998958802</v>
+      </c>
+      <c r="J52">
+        <v>0.5764402999921</v>
+      </c>
+      <c r="K52">
+        <v>0.629853166668908</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>13</v>
+      </c>
+      <c r="B53">
+        <v>100000000</v>
+      </c>
+      <c r="C53">
+        <v>4</v>
+      </c>
+      <c r="D53" t="s">
+        <v>15</v>
+      </c>
+      <c r="E53">
+        <v>0.44522756666992702</v>
+      </c>
+      <c r="F53">
+        <v>4.3149898139205098E-2</v>
+      </c>
+      <c r="G53">
+        <v>1.4146769288790499</v>
+      </c>
+      <c r="H53">
+        <v>0.49269719999574502</v>
+      </c>
+      <c r="I53">
+        <v>0.408382100009475</v>
+      </c>
+      <c r="J53">
+        <v>0.43460340000456199</v>
+      </c>
+      <c r="K53">
+        <v>0.629853166668908</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>13</v>
+      </c>
+      <c r="B54">
+        <v>100000000</v>
+      </c>
+      <c r="C54">
+        <v>5</v>
+      </c>
+      <c r="D54" t="s">
+        <v>15</v>
+      </c>
+      <c r="E54">
+        <v>0.45080863333229598</v>
+      </c>
+      <c r="F54">
+        <v>2.1607134569779501E-2</v>
+      </c>
+      <c r="G54">
+        <v>1.3971630534516299</v>
+      </c>
+      <c r="H54">
+        <v>0.42724370000360001</v>
+      </c>
+      <c r="I54">
+        <v>0.45549259999825098</v>
+      </c>
+      <c r="J54">
+        <v>0.46968959999503501</v>
+      </c>
+      <c r="K54">
+        <v>0.629853166668908</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>13</v>
+      </c>
+      <c r="B55">
+        <v>100000000</v>
+      </c>
+      <c r="C55">
+        <v>6</v>
+      </c>
+      <c r="D55" t="s">
+        <v>15</v>
+      </c>
+      <c r="E55">
+        <v>0.481060099996587</v>
+      </c>
+      <c r="F55">
+        <v>1.7193796162734101E-2</v>
+      </c>
+      <c r="G55">
+        <v>1.30930244822502</v>
+      </c>
+      <c r="H55">
+        <v>0.49539779999758998</v>
+      </c>
+      <c r="I55">
+        <v>0.48578449999331402</v>
+      </c>
+      <c r="J55">
+        <v>0.46199799999885699</v>
+      </c>
+      <c r="K55">
+        <v>0.629853166668908</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>13</v>
+      </c>
+      <c r="B56">
+        <v>100000000</v>
+      </c>
+      <c r="C56">
+        <v>7</v>
+      </c>
+      <c r="D56" t="s">
+        <v>15</v>
+      </c>
+      <c r="E56">
+        <v>0.50728569999531203</v>
+      </c>
+      <c r="F56">
+        <v>4.1341038724482401E-2</v>
+      </c>
+      <c r="G56">
+        <v>1.24161427510124</v>
+      </c>
+      <c r="H56">
+        <v>0.53467719999025498</v>
+      </c>
+      <c r="I56">
+        <v>0.52744790000724595</v>
+      </c>
+      <c r="J56">
+        <v>0.459731999988434</v>
+      </c>
+      <c r="K56">
+        <v>0.629853166668908</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>13</v>
+      </c>
+      <c r="B57">
+        <v>100000000</v>
+      </c>
+      <c r="C57">
+        <v>8</v>
+      </c>
+      <c r="D57" t="s">
+        <v>15</v>
+      </c>
+      <c r="E57">
+        <v>0.48672753333812502</v>
+      </c>
+      <c r="F57">
+        <v>3.6069502864706601E-2</v>
+      </c>
+      <c r="G57">
+        <v>1.2940569898505301</v>
+      </c>
+      <c r="H57">
+        <v>0.48682700000063001</v>
+      </c>
+      <c r="I57">
+        <v>0.52274720001150798</v>
+      </c>
+      <c r="J57">
+        <v>0.45060840000223801</v>
+      </c>
+      <c r="K57">
+        <v>0.629853166668908</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>13</v>
+      </c>
+      <c r="B58">
+        <v>1000000000</v>
+      </c>
+      <c r="C58">
+        <v>1</v>
+      </c>
+      <c r="D58" t="s">
+        <v>15</v>
+      </c>
+      <c r="E58">
+        <v>8.2424504000033796</v>
+      </c>
+      <c r="F58">
+        <v>0.34710810429007399</v>
+      </c>
+      <c r="G58">
+        <v>1</v>
+      </c>
+      <c r="H58">
+        <v>8.5039141000015608</v>
+      </c>
+      <c r="I58">
+        <v>8.3747995000012398</v>
+      </c>
+      <c r="J58">
+        <v>7.8486376000073497</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>13</v>
+      </c>
+      <c r="B59">
+        <v>1000000000</v>
+      </c>
+      <c r="C59">
+        <v>2</v>
+      </c>
+      <c r="D59" t="s">
+        <v>15</v>
+      </c>
+      <c r="E59">
+        <v>5.5658988333355701</v>
+      </c>
+      <c r="F59">
+        <v>8.5875190747178407E-2</v>
+      </c>
+      <c r="G59">
+        <v>1.4808839770204301</v>
+      </c>
+      <c r="H59">
+        <v>5.66356169999926</v>
+      </c>
+      <c r="I59">
+        <v>5.5022006000071997</v>
+      </c>
+      <c r="J59">
+        <v>5.5319342000002498</v>
+      </c>
+      <c r="K59">
+        <v>8.2424504000033796</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>13</v>
+      </c>
+      <c r="B60">
+        <v>1000000000</v>
+      </c>
+      <c r="C60">
+        <v>3</v>
+      </c>
+      <c r="D60" t="s">
+        <v>15</v>
+      </c>
+      <c r="E60">
+        <v>5.5213198333367401</v>
+      </c>
+      <c r="F60">
+        <v>0.85849718219488502</v>
+      </c>
+      <c r="G60">
+        <v>1.49284059768407</v>
+      </c>
+      <c r="H60">
+        <v>4.7187250999995696</v>
+      </c>
+      <c r="I60">
+        <v>5.4187336000031703</v>
+      </c>
+      <c r="J60">
+        <v>6.4265008000074797</v>
+      </c>
+      <c r="K60">
+        <v>8.2424504000033796</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>13</v>
+      </c>
+      <c r="B61">
+        <v>1000000000</v>
+      </c>
+      <c r="C61">
+        <v>4</v>
+      </c>
+      <c r="D61" t="s">
+        <v>15</v>
+      </c>
+      <c r="E61">
+        <v>5.6767926333365404</v>
+      </c>
+      <c r="F61">
+        <v>3.5173700666825701E-2</v>
+      </c>
+      <c r="G61">
+        <v>1.4519555200237899</v>
+      </c>
+      <c r="H61">
+        <v>5.7065953999990597</v>
+      </c>
+      <c r="I61">
+        <v>5.6857875999994496</v>
+      </c>
+      <c r="J61">
+        <v>5.6379949000111003</v>
+      </c>
+      <c r="K61">
+        <v>8.2424504000033796</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>13</v>
+      </c>
+      <c r="B62">
+        <v>1000000000</v>
+      </c>
+      <c r="C62">
+        <v>5</v>
+      </c>
+      <c r="D62" t="s">
+        <v>15</v>
+      </c>
+      <c r="E62">
+        <v>5.6010427000001002</v>
+      </c>
+      <c r="F62">
+        <v>0.128106510964724</v>
+      </c>
+      <c r="G62">
+        <v>1.47159213765737</v>
+      </c>
+      <c r="H62">
+        <v>5.4983750999963297</v>
+      </c>
+      <c r="I62">
+        <v>5.5601496000017496</v>
+      </c>
+      <c r="J62">
+        <v>5.7446034000022301</v>
+      </c>
+      <c r="K62">
+        <v>8.2424504000033796</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>13</v>
+      </c>
+      <c r="B63">
+        <v>1000000000</v>
+      </c>
+      <c r="C63">
+        <v>6</v>
+      </c>
+      <c r="D63" t="s">
+        <v>15</v>
+      </c>
+      <c r="E63">
+        <v>5.3453203333386501</v>
+      </c>
+      <c r="F63">
+        <v>0.59559661430159505</v>
+      </c>
+      <c r="G63">
+        <v>1.5419937227326399</v>
+      </c>
+      <c r="H63">
+        <v>6.0284435000066798</v>
+      </c>
+      <c r="I63">
+        <v>5.0726237000053498</v>
+      </c>
+      <c r="J63">
+        <v>4.9348938000039198</v>
+      </c>
+      <c r="K63">
+        <v>8.2424504000033796</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>13</v>
+      </c>
+      <c r="B64">
+        <v>1000000000</v>
+      </c>
+      <c r="C64">
+        <v>7</v>
+      </c>
+      <c r="D64" t="s">
+        <v>15</v>
+      </c>
+      <c r="E64">
+        <v>4.9262269666602698</v>
+      </c>
+      <c r="F64">
+        <v>0.299600232725515</v>
+      </c>
+      <c r="G64">
+        <v>1.67317715074572</v>
+      </c>
+      <c r="H64">
+        <v>5.26828839999507</v>
+      </c>
+      <c r="I64">
+        <v>4.7104102999874096</v>
+      </c>
+      <c r="J64">
+        <v>4.7999821999983396</v>
+      </c>
+      <c r="K64">
+        <v>8.2424504000033796</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>13</v>
+      </c>
+      <c r="B65">
+        <v>1000000000</v>
+      </c>
+      <c r="C65">
+        <v>8</v>
+      </c>
+      <c r="D65" t="s">
+        <v>15</v>
+      </c>
+      <c r="E65">
+        <v>4.4250023666730396</v>
+      </c>
+      <c r="F65">
+        <v>0.17193607611244199</v>
+      </c>
+      <c r="G65">
+        <v>1.86269965911916</v>
+      </c>
+      <c r="H65">
+        <v>4.6223673000058598</v>
+      </c>
+      <c r="I65">
+        <v>4.3449566000053803</v>
+      </c>
+      <c r="J65">
+        <v>4.3076832000078804</v>
+      </c>
+      <c r="K65">
+        <v>8.2424504000033796</v>
       </c>
     </row>
   </sheetData>

</xml_diff>